<commit_message>
Day 35: Complete portfolio summary and final validation
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>capital_allocation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +520,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -560,6 +570,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,6 +618,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -646,6 +666,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -691,6 +716,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -734,6 +764,11 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>Shareholder Returns / Debt Reduction</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -779,6 +814,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -824,6 +864,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -869,6 +914,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -912,6 +962,11 @@
       <c r="K11" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -957,6 +1012,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1000,6 +1060,11 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1045,6 +1110,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1088,6 +1158,11 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1133,6 +1208,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1176,6 +1256,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1219,6 +1304,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1262,6 +1352,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1305,6 +1400,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1348,6 +1448,11 @@
       <c r="K21" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -1393,6 +1498,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1438,6 +1548,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1481,6 +1596,11 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1526,6 +1646,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1571,6 +1696,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1616,6 +1746,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1661,6 +1796,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1706,6 +1846,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1749,6 +1894,11 @@
       <c r="K30" t="inlineStr">
         <is>
           <t>Shareholder Returns / Debt Reduction</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -1794,6 +1944,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1839,6 +1994,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1884,6 +2044,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1927,6 +2092,11 @@
       <c r="K34" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1972,6 +2142,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2015,6 +2190,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2058,6 +2238,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2103,6 +2288,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2146,6 +2336,11 @@
       <c r="K39" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2191,6 +2386,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2234,6 +2434,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2279,6 +2484,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2324,6 +2534,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2369,6 +2584,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2414,6 +2634,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2459,6 +2684,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2504,6 +2734,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2547,6 +2782,11 @@
       <c r="K48" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2592,6 +2832,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2635,6 +2880,11 @@
       <c r="K50" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2680,6 +2930,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2723,6 +2978,11 @@
       <c r="K52" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2768,6 +3028,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2811,6 +3076,11 @@
       <c r="K54" t="inlineStr">
         <is>
           <t>Shareholder Returns / Debt Reduction</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -2856,6 +3126,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2899,6 +3174,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2942,6 +3222,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2985,6 +3270,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3028,6 +3318,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3071,6 +3366,11 @@
       <c r="K60" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3116,6 +3416,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3159,6 +3464,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3202,6 +3512,11 @@
       <c r="K63" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3247,6 +3562,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3292,6 +3612,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3335,6 +3660,11 @@
       <c r="K66" t="inlineStr">
         <is>
           <t>Shareholder Returns / Debt Reduction</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3380,6 +3710,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3425,6 +3760,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3468,6 +3808,11 @@
       <c r="K69" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3513,6 +3858,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3556,6 +3906,11 @@
       <c r="K71" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3601,6 +3956,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3644,6 +4004,11 @@
       <c r="K73" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3689,6 +4054,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3732,6 +4102,11 @@
       <c r="K75" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3777,6 +4152,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3820,6 +4200,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3863,6 +4248,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3908,6 +4298,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3951,6 +4346,11 @@
       <c r="K80" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3996,6 +4396,11 @@
           <t>Distress Financing</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4041,6 +4446,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4086,6 +4496,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4129,6 +4544,11 @@
       <c r="K84" t="inlineStr">
         <is>
           <t>Shareholder Returns / Debt Reduction</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -4174,6 +4594,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4217,6 +4642,11 @@
       <c r="K86" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4262,6 +4692,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4307,6 +4742,11 @@
           <t>Shareholder Returns / Debt Reduction</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4352,6 +4792,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4397,6 +4842,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4440,6 +4890,11 @@
       <c r="K91" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4485,6 +4940,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4526,6 +4986,11 @@
       <c r="K93" t="inlineStr">
         <is>
           <t>Distress Financing</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
         </is>
       </c>
     </row>

</xml_diff>